<commit_message>
Regenerate sample evidence with authentic, realistic content
- Text notes: full multi-paragraph reports/statements instead of one-liners,
  with consistent names, badges, case numbers, and cross-references
- Images: detailed synthetic scene renders (gradient lighting, textured
  facades, forced-entry marks, evidence markers, film grain) instead of
  flat text-on-background cards
- Video: CCTV-style renders with timestamp/camera burn-in, grain, and
  moving person/vehicle silhouettes
- Audio: real synthesized speech via macOS say + afconvert (witness
  statement, dispatch call, detective voice memo) instead of sine tones,
  so Whisper/Groq transcription has actual spoken content
- Updated data/sample_evidence/README.md to describe the new content

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/sample_evidence/case-01-millbrook-heights/suspect_associates.xlsx
+++ b/data/sample_evidence/case-01-millbrook-heights/suspect_associates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Daniel Marsh</t>
+          <t>Daniel R. Marsh</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -446,7 +446,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>person of interest</t>
+          <t>person of interest, tool-mark/vehicle pattern match</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,41 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>seen in vehicle</t>
+          <t>seen in vehicle passenger seat by witness</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Carol Ann Whitfield</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>victim/complainant</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>reported incident, provided initial statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Harold Pruitt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>witness</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>provided statement re: vehicle and timeline</t>
         </is>
       </c>
     </row>

</xml_diff>